<commit_message>
revised CVE node properties listed in docs/cti-schema-target-2026-02.xlsx plus json test template files in schema-test/
</commit_message>
<xml_diff>
--- a/tmpl_gen/docs/cti-schema-target-2026-02.xlsx
+++ b/tmpl_gen/docs/cti-schema-target-2026-02.xlsx
@@ -148,7 +148,7 @@
     <t xml:space="preserve">cve:CVE</t>
   </si>
   <si>
-    <t xml:space="preserve">id, created, modified, title, affected, product, value, metrics, vectorString, baseScore, workarounds, exploits</t>
+    <t xml:space="preserve">id, created, modified, title, affected, affected_products, descriptions, metrics, cvss3_1_vectorString, cvss3_1_baseScore, cvss3_1_attackVector, workarounds, exploits</t>
   </si>
   <si>
     <t xml:space="preserve">capec:CAPEC</t>
@@ -367,6 +367,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -388,11 +389,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -466,51 +469,51 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -698,629 +701,629 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:I94"/>
-  <sheetFormatPr defaultColWidth="11.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="28.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.05"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="1"/>
-      <c r="F2" s="2" t="s">
+      <c r="D2" s="2"/>
+      <c r="F2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="E14" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="0" t="s">
+      <c r="E16" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="E17" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="D18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E18" s="0" t="s">
+      <c r="E18" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="D19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E19" s="0" t="s">
+      <c r="E19" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="D20" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="0" t="s">
+      <c r="E20" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="0" t="s">
+      <c r="D21" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="0" t="s">
+      <c r="E21" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="D22" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E22" s="0" t="s">
+      <c r="E22" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D23" s="0" t="s">
+      <c r="D23" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="0" t="s">
+      <c r="E23" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D24" s="0" t="s">
+      <c r="D24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E24" s="0" t="s">
+      <c r="E24" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="0" t="s">
+      <c r="D25" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E25" s="0" t="s">
+      <c r="E25" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="0" t="s">
+      <c r="D26" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E26" s="0" t="s">
+      <c r="E26" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="0" t="s">
+      <c r="D27" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E27" s="0" t="s">
+      <c r="E27" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="0" t="s">
+      <c r="D28" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E28" s="0" t="s">
+      <c r="E28" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D29" s="0" t="s">
+      <c r="D29" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E29" s="0" t="s">
+      <c r="E29" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E30" s="0" t="s">
+      <c r="E30" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C31" s="1" t="s">
+      <c r="C31" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D31" s="1"/>
-      <c r="E31" s="0" t="s">
+      <c r="D31" s="2"/>
+      <c r="E31" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D32" s="7"/>
-      <c r="E32" s="0" t="s">
+      <c r="D32" s="8"/>
+      <c r="E32" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D33" s="7"/>
-      <c r="E33" s="0" t="s">
+      <c r="D33" s="8"/>
+      <c r="E33" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D34" s="7"/>
-      <c r="E34" s="0" t="s">
+      <c r="D34" s="8"/>
+      <c r="E34" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C35" s="7" t="s">
+      <c r="C35" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="D35" s="7"/>
-      <c r="E35" s="0" t="s">
+      <c r="D35" s="8"/>
+      <c r="E35" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C36" s="7" t="s">
+      <c r="C36" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D36" s="7"/>
-      <c r="E36" s="0" t="s">
+      <c r="D36" s="8"/>
+      <c r="E36" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C37" s="7" t="s">
+      <c r="C37" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="7"/>
-      <c r="E37" s="0" t="s">
+      <c r="D37" s="8"/>
+      <c r="E37" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="D38" s="7"/>
-      <c r="E38" s="0" t="s">
+      <c r="D38" s="8"/>
+      <c r="E38" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C39" s="7" t="s">
+      <c r="C39" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="D39" s="7"/>
-      <c r="E39" s="0" t="s">
+      <c r="D39" s="8"/>
+      <c r="E39" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D40" s="7"/>
-      <c r="E40" s="0" t="s">
+      <c r="D40" s="8"/>
+      <c r="E40" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C41" s="7" t="s">
+      <c r="C41" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D41" s="7"/>
-      <c r="E41" s="0" t="s">
+      <c r="D41" s="8"/>
+      <c r="E41" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C42" s="7" t="s">
+      <c r="C42" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D42" s="7"/>
-      <c r="E42" s="0" t="s">
+      <c r="D42" s="8"/>
+      <c r="E42" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C43" s="7" t="s">
+      <c r="C43" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="D43" s="7"/>
-      <c r="E43" s="0" t="s">
+      <c r="D43" s="8"/>
+      <c r="E43" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C44" s="7" t="s">
+      <c r="C44" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="D44" s="7"/>
-      <c r="E44" s="0" t="s">
+      <c r="D44" s="8"/>
+      <c r="E44" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C45" s="7" t="s">
+      <c r="C45" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="D45" s="7"/>
-      <c r="E45" s="0" t="s">
+      <c r="D45" s="8"/>
+      <c r="E45" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C46" s="7" t="s">
+      <c r="C46" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D46" s="7"/>
-      <c r="E46" s="0" t="s">
+      <c r="D46" s="8"/>
+      <c r="E46" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C47" s="7" t="s">
+      <c r="C47" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="D47" s="7"/>
-      <c r="E47" s="0" t="s">
+      <c r="D47" s="8"/>
+      <c r="E47" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="0" t="s">
+      <c r="B48" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C48" s="8" t="s">
+      <c r="C48" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D48" s="8"/>
-      <c r="E48" s="0" t="s">
+      <c r="D48" s="9"/>
+      <c r="E48" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="0" t="s">
+      <c r="B49" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C49" s="8" t="s">
+      <c r="C49" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D49" s="8"/>
-      <c r="E49" s="0" t="s">
+      <c r="D49" s="9"/>
+      <c r="E49" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C50" s="9" t="s">
+      <c r="C50" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="D50" s="9"/>
-      <c r="E50" s="0" t="s">
+      <c r="D50" s="10"/>
+      <c r="E50" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="D51" s="9"/>
-      <c r="E51" s="0" t="s">
+      <c r="D51" s="10"/>
+      <c r="E51" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="36.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C52" s="9" t="s">
+      <c r="C52" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="D52" s="9"/>
-      <c r="E52" s="0" t="s">
+      <c r="D52" s="10"/>
+      <c r="E52" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C53" s="7" t="s">
+      <c r="C53" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D53" s="7"/>
-      <c r="E53" s="0" t="s">
+      <c r="D53" s="8"/>
+      <c r="E53" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C54" s="7" t="s">
+      <c r="C54" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="D54" s="7"/>
-      <c r="E54" s="0" t="s">
+      <c r="D54" s="8"/>
+      <c r="E54" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C55" s="7" t="s">
+      <c r="C55" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="D55" s="7"/>
-      <c r="E55" s="0" t="s">
+      <c r="D55" s="8"/>
+      <c r="E55" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="36.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C56" s="7" t="s">
+      <c r="C56" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D56" s="7"/>
-      <c r="E56" s="0" t="s">
+      <c r="D56" s="8"/>
+      <c r="E56" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C57" s="7" t="s">
+      <c r="C57" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D57" s="7"/>
-      <c r="E57" s="0" t="s">
+      <c r="D57" s="8"/>
+      <c r="E57" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C58" s="7" t="s">
+      <c r="C58" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="D58" s="7"/>
-      <c r="E58" s="0" t="s">
+      <c r="D58" s="8"/>
+      <c r="E58" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C59" s="7" t="s">
+      <c r="C59" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D59" s="7"/>
-      <c r="E59" s="0" t="s">
+      <c r="D59" s="8"/>
+      <c r="E59" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C60" s="9" t="s">
+      <c r="C60" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="D60" s="9"/>
-      <c r="E60" s="0" t="s">
+      <c r="D60" s="10"/>
+      <c r="E60" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C61" s="7" t="s">
+      <c r="C61" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D61" s="7"/>
-      <c r="E61" s="0" t="s">
+      <c r="D61" s="8"/>
+      <c r="E61" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C62" s="7" t="s">
+      <c r="C62" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D62" s="7"/>
-      <c r="E62" s="0" t="s">
+      <c r="D62" s="8"/>
+      <c r="E62" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="10"/>
-      <c r="B63" s="10"/>
-      <c r="C63" s="9" t="s">
+      <c r="A63" s="1"/>
+      <c r="B63" s="1"/>
+      <c r="C63" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="D63" s="9"/>
-      <c r="E63" s="0" t="s">
+      <c r="D63" s="10"/>
+      <c r="E63" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1329,7 +1332,7 @@
         <v>92</v>
       </c>
       <c r="D64" s="11"/>
-      <c r="E64" s="0" t="s">
+      <c r="E64" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1338,7 +1341,7 @@
         <v>93</v>
       </c>
       <c r="D65" s="11"/>
-      <c r="E65" s="0" t="s">
+      <c r="E65" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1347,7 +1350,7 @@
         <v>94</v>
       </c>
       <c r="D66" s="11"/>
-      <c r="E66" s="0" t="s">
+      <c r="E66" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1356,142 +1359,142 @@
         <v>95</v>
       </c>
       <c r="D67" s="11"/>
-      <c r="E67" s="0" t="s">
+      <c r="E67" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C68" s="9" t="s">
+      <c r="C68" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="D68" s="9"/>
-      <c r="E68" s="0" t="s">
+      <c r="D68" s="10"/>
+      <c r="E68" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C69" s="9" t="s">
+      <c r="C69" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="D69" s="9"/>
-      <c r="E69" s="0" t="s">
+      <c r="D69" s="10"/>
+      <c r="E69" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C70" s="9" t="s">
+      <c r="C70" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="D70" s="9"/>
-      <c r="E70" s="0" t="s">
+      <c r="D70" s="10"/>
+      <c r="E70" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C71" s="9" t="s">
+      <c r="C71" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="D71" s="9"/>
-      <c r="E71" s="0" t="s">
+      <c r="D71" s="10"/>
+      <c r="E71" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C72" s="9" t="s">
+      <c r="C72" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="D72" s="9"/>
-      <c r="E72" s="0" t="s">
+      <c r="D72" s="10"/>
+      <c r="E72" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="D73" s="9"/>
-      <c r="E73" s="0" t="s">
+      <c r="D73" s="10"/>
+      <c r="E73" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C74" s="9" t="s">
+      <c r="C74" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="D74" s="9"/>
-      <c r="E74" s="0" t="s">
+      <c r="D74" s="10"/>
+      <c r="E74" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C75" s="9" t="s">
+      <c r="C75" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="D75" s="9"/>
-      <c r="E75" s="0" t="s">
+      <c r="D75" s="10"/>
+      <c r="E75" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C76" s="9" t="s">
+      <c r="C76" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="D76" s="9"/>
-      <c r="E76" s="0" t="s">
+      <c r="D76" s="10"/>
+      <c r="E76" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C77" s="9" t="s">
+      <c r="C77" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="D77" s="9"/>
-      <c r="E77" s="0" t="s">
+      <c r="D77" s="10"/>
+      <c r="E77" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C78" s="9" t="s">
+      <c r="C78" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="D78" s="9"/>
-      <c r="E78" s="0" t="s">
+      <c r="D78" s="10"/>
+      <c r="E78" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C79" s="9" t="s">
+      <c r="C79" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="D79" s="9"/>
-      <c r="E79" s="0" t="s">
+      <c r="D79" s="10"/>
+      <c r="E79" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C80" s="9" t="s">
+      <c r="C80" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="D80" s="9"/>
-      <c r="E80" s="0" t="s">
+      <c r="D80" s="10"/>
+      <c r="E80" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C81" s="9" t="s">
+      <c r="C81" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="D81" s="9"/>
-      <c r="E81" s="0" t="s">
+      <c r="D81" s="10"/>
+      <c r="E81" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C82" s="9" t="s">
+      <c r="C82" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="D82" s="9"/>
-      <c r="E82" s="0" t="s">
+      <c r="D82" s="10"/>
+      <c r="E82" s="1" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
revised 02/2026 templates and schema doc
</commit_message>
<xml_diff>
--- a/tmpl_gen/docs/cti-schema-target-2026-02.xlsx
+++ b/tmpl_gen/docs/cti-schema-target-2026-02.xlsx
@@ -154,7 +154,23 @@
     <t xml:space="preserve">capec:CAPEC</t>
   </si>
   <si>
-    <t xml:space="preserve">id, name, status, consequences, created, modified, description, example_instances, likelihood_of_attack, mitigations, prerequisites, skills_required, severity, execution_flow</t>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="DejaVu Sans Mono"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">abstraction, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val=""/>
+        <family val="1"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">id, name, status, consequences, created, modified, description, example_instances, likelihood_of_attack, mitigations, prerequisites, skills_required, severity, execution_flow</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">en:goal</t>
@@ -362,7 +378,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -395,6 +411,17 @@
       <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="DejaVu Sans Mono"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val=""/>
+      <family val="1"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -464,7 +491,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -494,6 +521,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -922,7 +953,7 @@
       <c r="C21" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="8" t="s">
         <v>44</v>
       </c>
       <c r="E21" s="1" t="s">
@@ -1032,145 +1063,145 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="D32" s="8"/>
+      <c r="D32" s="9"/>
       <c r="E32" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D33" s="8"/>
+      <c r="D33" s="9"/>
       <c r="E33" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D34" s="8"/>
+      <c r="D34" s="9"/>
       <c r="E34" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="D35" s="8"/>
+      <c r="D35" s="9"/>
       <c r="E35" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D36" s="8"/>
+      <c r="D36" s="9"/>
       <c r="E36" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="8"/>
+      <c r="D37" s="9"/>
       <c r="E37" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="D38" s="8"/>
+      <c r="D38" s="9"/>
       <c r="E38" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D39" s="8"/>
+      <c r="D39" s="9"/>
       <c r="E39" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C40" s="8" t="s">
+      <c r="C40" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D40" s="8"/>
+      <c r="D40" s="9"/>
       <c r="E40" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C41" s="8" t="s">
+      <c r="C41" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D41" s="8"/>
+      <c r="D41" s="9"/>
       <c r="E41" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C42" s="8" t="s">
+      <c r="C42" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D42" s="8"/>
+      <c r="D42" s="9"/>
       <c r="E42" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C43" s="8" t="s">
+      <c r="C43" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="D43" s="8"/>
+      <c r="D43" s="9"/>
       <c r="E43" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C44" s="8" t="s">
+      <c r="C44" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D44" s="8"/>
+      <c r="D44" s="9"/>
       <c r="E44" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C45" s="8" t="s">
+      <c r="C45" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="D45" s="8"/>
+      <c r="D45" s="9"/>
       <c r="E45" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C46" s="8" t="s">
+      <c r="C46" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="D46" s="8"/>
+      <c r="D46" s="9"/>
       <c r="E46" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C47" s="8" t="s">
+      <c r="C47" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D47" s="8"/>
+      <c r="D47" s="9"/>
       <c r="E47" s="1" t="s">
         <v>11</v>
       </c>
@@ -1179,10 +1210,10 @@
       <c r="B48" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C48" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="D48" s="9"/>
+      <c r="D48" s="10"/>
       <c r="E48" s="1" t="s">
         <v>11</v>
       </c>
@@ -1191,127 +1222,127 @@
       <c r="B49" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="D49" s="9"/>
+      <c r="D49" s="10"/>
       <c r="E49" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C50" s="10" t="s">
+      <c r="C50" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="D50" s="10"/>
+      <c r="D50" s="11"/>
       <c r="E50" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C51" s="10" t="s">
+      <c r="C51" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="D51" s="10"/>
+      <c r="D51" s="11"/>
       <c r="E51" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="36.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C52" s="10" t="s">
+      <c r="C52" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="D52" s="10"/>
+      <c r="D52" s="11"/>
       <c r="E52" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C53" s="8" t="s">
+      <c r="C53" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="D53" s="8"/>
+      <c r="D53" s="9"/>
       <c r="E53" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C54" s="8" t="s">
+      <c r="C54" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="D54" s="8"/>
+      <c r="D54" s="9"/>
       <c r="E54" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C55" s="8" t="s">
+      <c r="C55" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="D55" s="8"/>
+      <c r="D55" s="9"/>
       <c r="E55" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="36.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C56" s="8" t="s">
+      <c r="C56" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="D56" s="8"/>
+      <c r="D56" s="9"/>
       <c r="E56" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C57" s="8" t="s">
+      <c r="C57" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="D57" s="8"/>
+      <c r="D57" s="9"/>
       <c r="E57" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C58" s="8" t="s">
+      <c r="C58" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="D58" s="8"/>
+      <c r="D58" s="9"/>
       <c r="E58" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C59" s="8" t="s">
+      <c r="C59" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="D59" s="8"/>
+      <c r="D59" s="9"/>
       <c r="E59" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C60" s="10" t="s">
+      <c r="C60" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="D60" s="10"/>
+      <c r="D60" s="11"/>
       <c r="E60" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C61" s="8" t="s">
+      <c r="C61" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D61" s="8"/>
+      <c r="D61" s="9"/>
       <c r="E61" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C62" s="8" t="s">
+      <c r="C62" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="D62" s="8"/>
+      <c r="D62" s="9"/>
       <c r="E62" s="1" t="s">
         <v>11</v>
       </c>
@@ -1319,192 +1350,192 @@
     <row r="63" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
-      <c r="C63" s="10" t="s">
+      <c r="C63" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="D63" s="10"/>
+      <c r="D63" s="11"/>
       <c r="E63" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C64" s="11" t="s">
+      <c r="C64" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D64" s="11"/>
+      <c r="D64" s="12"/>
       <c r="E64" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C65" s="11" t="s">
+      <c r="C65" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="D65" s="11"/>
+      <c r="D65" s="12"/>
       <c r="E65" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C66" s="11" t="s">
+      <c r="C66" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="D66" s="11"/>
+      <c r="D66" s="12"/>
       <c r="E66" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C67" s="11" t="s">
+      <c r="C67" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="D67" s="11"/>
+      <c r="D67" s="12"/>
       <c r="E67" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C68" s="10" t="s">
+      <c r="C68" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="D68" s="10"/>
+      <c r="D68" s="11"/>
       <c r="E68" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C69" s="10" t="s">
+      <c r="C69" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="D69" s="10"/>
+      <c r="D69" s="11"/>
       <c r="E69" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C70" s="10" t="s">
+      <c r="C70" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="D70" s="10"/>
+      <c r="D70" s="11"/>
       <c r="E70" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C71" s="10" t="s">
+      <c r="C71" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D71" s="10"/>
+      <c r="D71" s="11"/>
       <c r="E71" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C72" s="10" t="s">
+      <c r="C72" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="D72" s="10"/>
+      <c r="D72" s="11"/>
       <c r="E72" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C73" s="10" t="s">
+      <c r="C73" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D73" s="10"/>
+      <c r="D73" s="11"/>
       <c r="E73" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C74" s="10" t="s">
+      <c r="C74" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D74" s="10"/>
+      <c r="D74" s="11"/>
       <c r="E74" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C75" s="10" t="s">
+      <c r="C75" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="D75" s="10"/>
+      <c r="D75" s="11"/>
       <c r="E75" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C76" s="10" t="s">
+      <c r="C76" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="D76" s="10"/>
+      <c r="D76" s="11"/>
       <c r="E76" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C77" s="10" t="s">
+      <c r="C77" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="D77" s="10"/>
+      <c r="D77" s="11"/>
       <c r="E77" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C78" s="10" t="s">
+      <c r="C78" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="D78" s="10"/>
+      <c r="D78" s="11"/>
       <c r="E78" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C79" s="10" t="s">
+      <c r="C79" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="D79" s="10"/>
+      <c r="D79" s="11"/>
       <c r="E79" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C80" s="10" t="s">
+      <c r="C80" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="D80" s="10"/>
+      <c r="D80" s="11"/>
       <c r="E80" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C81" s="10" t="s">
+      <c r="C81" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="D81" s="10"/>
+      <c r="D81" s="11"/>
       <c r="E81" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C82" s="10" t="s">
+      <c r="C82" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="D82" s="10"/>
+      <c r="D82" s="11"/>
       <c r="E82" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C83" s="12"/>
-      <c r="D83" s="12"/>
+      <c r="C83" s="13"/>
+      <c r="D83" s="13"/>
     </row>
     <row r="84" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C84" s="12"/>
-      <c r="D84" s="12"/>
+      <c r="C84" s="13"/>
+      <c r="D84" s="13"/>
     </row>
     <row r="85" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="86" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
added EPSS to schema doc and xls summary
</commit_message>
<xml_diff>
--- a/tmpl_gen/docs/cti-schema-target-2026-02.xlsx
+++ b/tmpl_gen/docs/cti-schema-target-2026-02.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="111">
   <si>
     <t xml:space="preserve">Color Coding:</t>
   </si>
@@ -53,9 +53,6 @@
   </si>
   <si>
     <t xml:space="preserve">created, description, external_references, id, kill_chain_phases, mitre_id, modified, name, type, x_mitre_data_sources, x_mitre_deprecated, x_mitre_detection, x_mitre_domains, x_mitre_is_subtechnique, x_mitre_platforms, x_mitre_version,  x_mitre_attack_spec_version</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t xml:space="preserve">campaign</t>
@@ -159,13 +156,14 @@
         <sz val="9"/>
         <rFont val="DejaVu Sans Mono"/>
         <family val="1"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">abstraction, </t>
     </r>
     <r>
       <rPr>
         <sz val="12"/>
-        <rFont val=""/>
+        <rFont val="DejaVu Sans Mono"/>
         <family val="1"/>
         <charset val="1"/>
       </rPr>
@@ -212,6 +210,15 @@
     <t xml:space="preserve">cveID, vendorProject, product, vulnerabilityName, dateAdded, shortDescription, requiredAction, dueDate, knownRansomwareCampaignUse, notes, cwes</t>
   </si>
   <si>
+    <t xml:space="preserve">epss:EPSS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cve, epss, percentile</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
     <t xml:space="preserve">Relationships</t>
   </si>
   <si>
@@ -263,15 +270,6 @@
     <t xml:space="preserve">tool - uses - attack-pattern</t>
   </si>
   <si>
-    <t xml:space="preserve">deprecated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">x-mitre-data-component - detects - attack-pattern</t>
-  </si>
-  <si>
-    <t xml:space="preserve">x-mitre-data-component - belongs_to - x-mitre-data-source</t>
-  </si>
-  <si>
     <t xml:space="preserve">x-mitre-detection-strategy - detects - attack-pattern</t>
   </si>
   <si>
@@ -369,6 +367,9 @@
   </si>
   <si>
     <t xml:space="preserve">en:vulnerability - with_tactic - en:attack_tactic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epss:EPSS - scores - cve:CVE</t>
   </si>
 </sst>
 </file>
@@ -417,10 +418,11 @@
       <sz val="9"/>
       <name val="DejaVu Sans Mono"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
-      <name val=""/>
+      <name val="DejaVu Sans Mono"/>
       <family val="1"/>
       <charset val="1"/>
     </font>
@@ -491,7 +493,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -520,27 +522,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -731,7 +717,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:I94"/>
+  <dimension ref="A2:I93"/>
   <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="28.11"/>
@@ -777,776 +763,663 @@
       <c r="D5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="E5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="E6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="E7" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="E8" s="1"/>
     </row>
     <row r="9" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="E9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="E10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="E11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C12" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C13" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C14" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C15" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C17" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C17" s="7" t="s">
+      <c r="D17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="E17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="D18" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="E18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C19" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C20" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C20" s="7" t="s">
+      <c r="D20" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C21" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C21" s="7" t="s">
+      <c r="D21" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C22" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C23" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C24" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D23" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C25" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D24" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C26" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C27" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E27" s="1"/>
+    </row>
+    <row r="28" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C28" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C28" s="5" t="s">
+      <c r="D28" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="E28" s="1"/>
+    </row>
+    <row r="29" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C29" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C29" s="7" t="s">
+      <c r="D29" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C30" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E30" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="D30" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E30" s="1"/>
     </row>
     <row r="31" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C31" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D31" s="2"/>
       <c r="E31" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C32" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="D32" s="9"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C32" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D32" s="2"/>
       <c r="E32" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C33" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="D33" s="9"/>
+      <c r="C33" s="8" t="s">
+        <v>61</v>
+      </c>
       <c r="E33" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C34" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="D34" s="9"/>
+      <c r="C34" s="8" t="s">
+        <v>62</v>
+      </c>
       <c r="E34" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C35" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="D35" s="9"/>
+      <c r="C35" s="8" t="s">
+        <v>63</v>
+      </c>
       <c r="E35" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C36" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="D36" s="9"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C36" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="E36" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C37" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="D37" s="9"/>
+      <c r="C37" s="8" t="s">
+        <v>65</v>
+      </c>
       <c r="E37" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C38" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D38" s="9"/>
+      <c r="C38" s="8" t="s">
+        <v>66</v>
+      </c>
       <c r="E38" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C39" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="D39" s="9"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C39" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="E39" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C40" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D40" s="9"/>
+      <c r="C40" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="E40" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C41" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="D41" s="9"/>
+      <c r="C41" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="E41" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C42" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D42" s="9"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C42" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="E42" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C43" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D43" s="9"/>
+      <c r="C43" s="8" t="s">
+        <v>71</v>
+      </c>
       <c r="E43" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C44" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="D44" s="9"/>
+      <c r="C44" s="8" t="s">
+        <v>72</v>
+      </c>
       <c r="E44" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C45" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="D45" s="9"/>
+      <c r="C45" s="8" t="s">
+        <v>73</v>
+      </c>
       <c r="E45" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C46" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="D46" s="9"/>
+      <c r="C46" s="8" t="s">
+        <v>74</v>
+      </c>
       <c r="E46" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C47" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D47" s="9"/>
+      <c r="C47" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="E47" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C48" s="10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C48" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="D48" s="10"/>
       <c r="E48" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C49" s="10" t="s">
+      <c r="C49" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D49" s="10"/>
       <c r="E49" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C50" s="11" t="s">
+      <c r="C50" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="D50" s="11"/>
       <c r="E50" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C51" s="11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="36.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C51" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="D51" s="11"/>
       <c r="E51" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="36.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C52" s="11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C52" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="D52" s="11"/>
       <c r="E52" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D53" s="9"/>
       <c r="E53" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C54" s="9" t="s">
+      <c r="C54" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="D54" s="9"/>
       <c r="E54" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C55" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="36.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C55" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="D55" s="9"/>
       <c r="E55" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="36.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C56" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C56" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D56" s="9"/>
       <c r="E56" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C57" s="9" t="s">
+      <c r="C57" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D57" s="9"/>
       <c r="E57" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C58" s="9" t="s">
+      <c r="C58" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="D58" s="9"/>
       <c r="E58" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C59" s="9" t="s">
+      <c r="C59" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D59" s="9"/>
       <c r="E59" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C60" s="11" t="s">
+      <c r="C60" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="D60" s="11"/>
       <c r="E60" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C61" s="9" t="s">
+      <c r="C61" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D61" s="9"/>
       <c r="E61" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C62" s="9" t="s">
+      <c r="A62" s="1"/>
+      <c r="B62" s="1"/>
+      <c r="C62" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D62" s="9"/>
       <c r="E62" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="1"/>
-      <c r="B63" s="1"/>
-      <c r="C63" s="11" t="s">
+      <c r="C63" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D63" s="11"/>
       <c r="E63" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C64" s="12" t="s">
+      <c r="C64" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="D64" s="12"/>
       <c r="E64" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C65" s="12" t="s">
+      <c r="C65" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="D65" s="12"/>
       <c r="E65" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C66" s="12" t="s">
+      <c r="C66" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="D66" s="12"/>
       <c r="E66" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C67" s="12" t="s">
+      <c r="C67" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="D67" s="12"/>
       <c r="E67" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C68" s="11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C68" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="D68" s="11"/>
       <c r="E68" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C69" s="11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C69" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D69" s="11"/>
       <c r="E69" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C70" s="11" t="s">
+      <c r="C70" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="D70" s="11"/>
       <c r="E70" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C71" s="11" t="s">
+      <c r="C71" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="D71" s="11"/>
       <c r="E71" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C72" s="11" t="s">
+      <c r="C72" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D72" s="11"/>
       <c r="E72" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C73" s="11" t="s">
+      <c r="C73" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="D73" s="11"/>
       <c r="E73" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C74" s="11" t="s">
+      <c r="C74" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="D74" s="11"/>
       <c r="E74" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C75" s="11" t="s">
+      <c r="C75" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="D75" s="11"/>
       <c r="E75" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C76" s="11" t="s">
+      <c r="C76" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="D76" s="11"/>
       <c r="E76" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C77" s="11" t="s">
+      <c r="C77" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="D77" s="11"/>
       <c r="E77" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C78" s="11" t="s">
+      <c r="C78" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D78" s="11"/>
       <c r="E78" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C79" s="11" t="s">
+      <c r="C79" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D79" s="11"/>
       <c r="E79" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C80" s="11" t="s">
+      <c r="C80" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="D80" s="11"/>
       <c r="E80" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C81" s="11" t="s">
+      <c r="C81" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D81" s="11"/>
       <c r="E81" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C82" s="11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C82" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="D82" s="11"/>
-      <c r="E82" s="1" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="83" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C83" s="13"/>
-      <c r="D83" s="13"/>
-    </row>
-    <row r="84" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C84" s="13"/>
-      <c r="D84" s="13"/>
-    </row>
+      <c r="C83" s="9"/>
+      <c r="D83" s="9"/>
+    </row>
+    <row r="84" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="85" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="86" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="87" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="88" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="89" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="90" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="90" customFormat="false" ht="32.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="91" customFormat="false" ht="32.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="92" customFormat="false" ht="32.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="93" customFormat="false" ht="32.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="94" customFormat="false" ht="32.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>